<commit_message>
volume and flow modification
</commit_message>
<xml_diff>
--- a/resources/data_import.xlsx
+++ b/resources/data_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1AC7139-7A3D-438C-B447-3C808802A693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6A2AAC-6954-4C53-84E7-6FABB6C2F3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
@@ -635,10 +635,10 @@
         <v>7200</v>
       </c>
       <c r="E2" s="5">
-        <v>43200</v>
+        <v>23000</v>
       </c>
       <c r="F2" s="5">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1">
         <v>4</v>
@@ -1057,10 +1057,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="B2" s="8">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="C2" s="1">
         <v>0.1</v>

</xml_diff>

<commit_message>
UI simulation duration conversion
</commit_message>
<xml_diff>
--- a/resources/data_import.xlsx
+++ b/resources/data_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6A2AAC-6954-4C53-84E7-6FABB6C2F3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0536BE1F-645A-45B0-BB9B-DFD29E9FB3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>Période d'entrée enzyme</t>
   </si>
   <si>
-    <t>Durée totale de simulation</t>
-  </si>
-  <si>
     <t>Pas de temps</t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>Période d'agitation du va et vient de R1</t>
   </si>
   <si>
-    <t>Période d'entrée de repas</t>
-  </si>
-  <si>
     <t>Viscosité</t>
   </si>
   <si>
@@ -120,6 +114,12 @@
   </si>
   <si>
     <t>Débit d'entrée de repas ml/min</t>
+  </si>
+  <si>
+    <t>Durée totale de simulation (min)</t>
+  </si>
+  <si>
+    <t>Période d'entrée de repas (min)</t>
   </si>
 </sst>
 </file>
@@ -600,10 +600,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -612,18 +612,18 @@
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="5">
         <v>50</v>
@@ -635,7 +635,7 @@
         <v>7200</v>
       </c>
       <c r="E2" s="5">
-        <v>23000</v>
+        <v>420</v>
       </c>
       <c r="F2" s="5">
         <v>15</v>
@@ -713,36 +713,36 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="8">
         <v>2</v>
@@ -771,7 +771,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="5">
         <v>10</v>
@@ -969,13 +969,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1043,16 +1043,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1060,7 +1060,7 @@
         <v>30</v>
       </c>
       <c r="B2" s="8">
-        <v>900</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1">
         <v>0.1</v>

</xml_diff>

<commit_message>
export modif : second to minute
</commit_message>
<xml_diff>
--- a/resources/data_import.xlsx
+++ b/resources/data_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED8A228-4B9B-4A9A-B306-EF079BCAFBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0A588B-E288-4B24-A08C-8BC334C4EFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -632,10 +632,10 @@
         <v>7200</v>
       </c>
       <c r="E2" s="5">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="F2" s="5">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="G2" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
Adding TR3 : reciprocating pump
</commit_message>
<xml_diff>
--- a/resources/data_import.xlsx
+++ b/resources/data_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1509DE8C-25D1-4925-B17E-4C740DA9A7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45DE5DB-BA5F-486E-B045-D3C139FCA8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="4" activeTab="5" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -260,15 +260,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -603,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F695C7B3-19CB-4070-9BD5-C34B803C5B05}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" customWidth="1"/>
@@ -616,7 +612,7 @@
     <col min="8" max="8" width="21.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -635,10 +631,8 @@
       <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -652,63 +646,51 @@
         <v>7200</v>
       </c>
       <c r="E2" s="4">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="F2" s="4">
         <v>60</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-    </row>
-    <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -735,66 +717,66 @@
       <c r="C1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
+      <c r="A2" s="9">
         <v>2.0833333333333333E-3</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>6.2500000000000003E-3</v>
       </c>
       <c r="C2" s="1">
         <v>4</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="4">
         <f>(B2-A2)*1440*C2</f>
         <v>24.000000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="11">
+      <c r="A3" s="10">
         <v>6.2500000000000003E-3</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>5.1388888888888887E-2</v>
       </c>
       <c r="C3" s="1">
         <v>7</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="4">
         <f t="shared" ref="D3:D5" si="0">(B3-A3)*1440*C3</f>
         <v>455</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
+      <c r="A4" s="10">
         <v>5.1388888888888887E-2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <v>7.2222222222222215E-2</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="4">
         <f t="shared" si="0"/>
         <v>119.99999999999997</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12">
+      <c r="A5" s="11">
         <v>7.2222222222222215E-2</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="11">
         <v>8.611111111111111E-2</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="5">
         <f t="shared" si="0"/>
         <v>60.000000000000021</v>
       </c>
@@ -806,7 +788,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{279F26CD-147B-4DCD-93E9-48B7B14504DF}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -814,7 +796,7 @@
     <col min="3" max="3" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>21</v>
       </c>
@@ -824,151 +806,63 @@
       <c r="C1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
         <v>1.2500000000000001E-2</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>2.9861111111111113E-2</v>
       </c>
       <c r="C2" s="1">
         <v>9</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="4">
         <f>(B2-A2)*1440*C2</f>
         <v>225</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="11">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
         <v>2.9861111111111113E-2</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>5.0694444444444445E-2</v>
       </c>
       <c r="C3" s="1">
         <v>7</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="4">
         <f>(B3-A3)*1440*C3</f>
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11">
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="10">
         <v>5.0694444444444445E-2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <v>0.20833333333333334</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="5">
         <f>(B4-A4)*1440*C4</f>
         <v>1135</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1257,7 +1151,7 @@
       </c>
       <c r="D2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>4300</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1415,7 +1309,7 @@
         <v>0.125</v>
       </c>
       <c r="C4">
-        <v>700</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
bug fixes: excel export + TR3 volume evolution fix
</commit_message>
<xml_diff>
--- a/resources/data_import.xlsx
+++ b/resources/data_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45DE5DB-BA5F-486E-B045-D3C139FCA8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329CE6B2-1C95-4861-93F9-4FF8E9C48168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
@@ -646,10 +646,10 @@
         <v>7200</v>
       </c>
       <c r="E2" s="4">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="F2" s="4">
-        <v>60</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>4100</v>
+        <v>400</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1285,7 +1285,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="C2">
-        <v>1500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1297,7 +1297,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C3">
-        <v>1700</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1309,7 +1309,7 @@
         <v>0.125</v>
       </c>
       <c r="C4">
-        <v>500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1321,7 +1321,7 @@
         <v>0.15625</v>
       </c>
       <c r="C5">
-        <v>400</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>